<commit_message>
eliminacion de vacaciones supervisor
</commit_message>
<xml_diff>
--- a/BBDD_empleados.xlsx
+++ b/BBDD_empleados.xlsx
@@ -855,10 +855,10 @@
         <v>14</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -959,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="18"/>
   <cols>
     <col width="12.3984375" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -2595,6 +2595,88 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>14</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>04/06/2026</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>04/07/2026</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Rechazada</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>falta personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>12</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>04/06/2026</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>6</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Solicitud aprobada</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
incorporacion de manual de usuario, actualizacion con cambios y mejoras readme, version final del código del chat bot vacaciones
</commit_message>
<xml_diff>
--- a/BBDD_empleados.xlsx
+++ b/BBDD_empleados.xlsx
@@ -739,10 +739,10 @@
         <v>21</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -855,10 +855,10 @@
         <v>14</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14">
@@ -959,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.796875" defaultRowHeight="18"/>
   <cols>
     <col width="12.3984375" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -2600,7 +2600,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -2609,20 +2609,20 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>04/07/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Rechazada</t>
+          <t>Aprobada</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2631,47 +2631,6 @@
         </is>
       </c>
       <c r="I45" t="inlineStr">
-        <is>
-          <t>falta personal</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" t="n">
-        <v>12</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>04/06/2026</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>05/06/2026</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>10/06/2026</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>6</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Aprobada</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Supervisor</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
         <is>
           <t>Solicitud aprobada</t>
         </is>

</xml_diff>